<commit_message>
Añadir columna Caja al inventario
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -426,19 +426,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -449,45 +450,50 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Caja</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Marca</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Modelo</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Nº de serie</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Procesador</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>RAM</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Almacenamiento</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Pantalla</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>

</xml_diff>

<commit_message>
Inventario: Caja 1 - Dell Latitude 3540
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,6 +29,9 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="3">
@@ -56,11 +59,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -499,6 +503,43 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Dell</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Latitude 3540 (Reg. P170G)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>4YLL214</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>15,6"</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Service Tag 4YLL214 · Express Code 10799233672 · Fab. 2024</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Inventario: Caja 1 - Dell Latitude 3550
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -540,6 +540,43 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Dell</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Latitude 3550</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>20FBX14</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>15,6"</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Service Tag 20FBX14 · Express Code 4379314936 · Fab. 2024</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Inventario: Caja 1 - Dell Latitude 3540 CYLL214
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -577,6 +577,43 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Dell</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Latitude 3540 (Reg. P170G)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>CYLL214</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>15,6"</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Service Tag CYLL214 · Express Code 28213492360 · Fab. 2024</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Inventario: Caja 1 - Dell Latitude 3540 JXLL214
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -614,6 +614,43 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Dell</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Latitude 3540 (Reg. P170G)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>JXLL214</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>15,6"</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Service Tag JXLL214 · Express Code 43390502536 · Fab. 2024</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Inventario: Caja 1 - Dell Latitude 3540 3PGYT04
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -651,6 +651,43 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Dell</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Latitude 3540 (Reg. P170G)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>3PGYT04</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>15,6"</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Service Tag 3PGYT04 · Express Code 8070499156 · Fab. 2024</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Inventario: Caja 1 - Dell Latitude 3550 DZDBX14
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -688,6 +688,43 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Dell</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Latitude 3550 (Reg. P170G)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>DZDBX14</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>15,6"</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Service Tag DZDBX14 · Express Code 30436877560 · Fab. 2024</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Inventario: Caja 1 - Dell Latitude 3540 DSLVMX3
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -725,6 +725,43 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Dell</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Latitude 3540</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>DSLVMX3</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>15,6"</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Service Tag DSLVMX3 · Express Code 30027971271 · Fab. 2023</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Inventario: DSLVMX3 movido a caja Renting
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -729,8 +729,10 @@
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="n">
-        <v>1</v>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Renting</t>
+        </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Inventario: specs Latitude 3540 y lista de renting
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventario" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lista Renting" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,7 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#,##0.00 €"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -59,12 +62,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -525,9 +530,21 @@
           <t>4YLL214</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Intel Core i7-1355U</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>512 GB SSD</t>
+        </is>
+      </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
           <t>15,6"</t>
@@ -536,7 +553,7 @@
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Service Tag 4YLL214 · Express Code 10799233672 · Fab. 2024</t>
+          <t>Service Tag 4YLL214 · Express Code 10799233672 · Fab. 2024 · W11 Pro · Specs según albarán renting (modelo 3540)</t>
         </is>
       </c>
     </row>
@@ -599,9 +616,21 @@
           <t>CYLL214</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Intel Core i7-1355U</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>512 GB SSD</t>
+        </is>
+      </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>15,6"</t>
@@ -610,7 +639,7 @@
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Service Tag CYLL214 · Express Code 28213492360 · Fab. 2024</t>
+          <t>Service Tag CYLL214 · Express Code 28213492360 · Fab. 2024 · W11 Pro · Specs según albarán renting (modelo 3540)</t>
         </is>
       </c>
     </row>
@@ -636,9 +665,21 @@
           <t>JXLL214</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Intel Core i7-1355U</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>512 GB SSD</t>
+        </is>
+      </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
           <t>15,6"</t>
@@ -647,7 +688,7 @@
       <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Service Tag JXLL214 · Express Code 43390502536 · Fab. 2024</t>
+          <t>Service Tag JXLL214 · Express Code 43390502536 · Fab. 2024 · W11 Pro · Specs según albarán renting (modelo 3540)</t>
         </is>
       </c>
     </row>
@@ -673,9 +714,21 @@
           <t>3PGYT04</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Intel Core i7-1355U</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>512 GB SSD</t>
+        </is>
+      </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
           <t>15,6"</t>
@@ -684,7 +737,7 @@
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Service Tag 3PGYT04 · Express Code 8070499156 · Fab. 2024</t>
+          <t>Service Tag 3PGYT04 · Express Code 8070499156 · Fab. 2024 · W11 Pro · Specs según albarán renting (modelo 3540)</t>
         </is>
       </c>
     </row>
@@ -749,9 +802,21 @@
           <t>DSLVMX3</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Intel Core i7-1355U</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>512 GB SSD</t>
+        </is>
+      </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
           <t>15,6"</t>
@@ -760,7 +825,125 @@
       <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Service Tag DSLVMX3 · Express Code 30027971271 · Fab. 2023</t>
+          <t>Service Tag DSLVMX3 · Express Code 30027971271 · Fab. 2023 · W11 Pro · Specs según albarán renting (modelo 3540)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Nº de serie</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Importe venta unitario</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>DSLVMX3</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Dell Latitude 3540 i7-1355U, 16GB, 512GB, 15,6" W11 Pro, 1 año garantía</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>1509</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>1MS1KX3</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Dell Latitude 3540 i7-1355U, 16GB, 512GB, 15,6" W11 Pro, 1 año garantía</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>1509</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>1VLVMX3</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Dell Latitude 3540 i7-1355U, 16GB, 512GB, 15,6" W11 Pro, 1 año garantía</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>1509</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2SLVMX3</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Dell Latitude 3540 i7-1355U, 16GB, 512GB, 15,6" W11 Pro, 1 año garantía</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>1509</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>4JS1KX3</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Dell Latitude 3540 i7-1355U, 16GB, 512GB, 15,6" W11 Pro, 1 año garantía</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>1509</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Nota: en la captura '1MS1KX3' y '4JS1KX3' podrían leerse con 5 en vez de S (1M51KX3 / 4J51KX3).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inventario: Caja 1 - Dell Latitude 3550 3WDBX14
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -826,6 +826,59 @@
       <c r="K8" s="2" t="inlineStr">
         <is>
           <t>Service Tag DSLVMX3 · Express Code 30027971271 · Fab. 2023 · W11 Pro · Specs según albarán renting (modelo 3540)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Dell</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Latitude 3550 (Reg. P170G)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>3WDBX14</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Intel Core i7-1355U (13ª gen)</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>512 GB SSD NVMe (Micron 2400)</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>15,6"</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Arranca OK</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Service Tag 3WDBX14 · Express Code 8487655672 · Fab. 2024 · Specs vistas en Administrador de tareas · W11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inventario: specs Latitude 3550
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -579,9 +579,21 @@
           <t>20FBX14</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Intel Core i7-1355U (13ª gen)</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>512 GB SSD NVMe</t>
+        </is>
+      </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
           <t>15,6"</t>
@@ -590,7 +602,7 @@
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Service Tag 20FBX14 · Express Code 4379314936 · Fab. 2024</t>
+          <t>Service Tag 20FBX14 · Express Code 4379314936 · Fab. 2024 · Specs según indicación (igual que 3WDBX14)</t>
         </is>
       </c>
     </row>
@@ -763,9 +775,21 @@
           <t>DZDBX14</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Intel Core i7-1355U (13ª gen)</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>512 GB SSD NVMe</t>
+        </is>
+      </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
           <t>15,6"</t>
@@ -774,7 +798,7 @@
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Service Tag DZDBX14 · Express Code 30436877560 · Fab. 2024</t>
+          <t>Service Tag DZDBX14 · Express Code 30436877560 · Fab. 2024 · Specs según indicación (igual que 3WDBX14)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inventario: Caja 1 - Dell Latitude 3540 7NGYT04
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -903,6 +903,55 @@
       <c r="K9" s="2" t="inlineStr">
         <is>
           <t>Service Tag 3WDBX14 · Express Code 8487655672 · Fab. 2024 · Specs vistas en Administrador de tareas · W11</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Dell</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Latitude 3540 (Reg. P170G)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>7NGYT04</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Intel Core i7-1355U</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>512 GB SSD</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>15,6"</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Service Tag 7NGYT04 · Express Code 16666996148 · Fab. 2024 · W11 Pro · Specs según albarán renting (modelo 3540)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inventario: Caja 1 - Dell Latitude 3540 6ZLL214
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -952,6 +952,55 @@
       <c r="K10" s="2" t="inlineStr">
         <is>
           <t>Service Tag 7NGYT04 · Express Code 16656696148 · Fab. 2024 · W11 Pro · Specs según albarán renting (modelo 3540)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Dell</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Latitude 3540 (Reg. P170G)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>6ZLL214</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Intel Core i7-1355U</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>512 GB SSD</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>15,6"</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Service Tag 6ZLL214 · Express Code 15213264520 · Fab. 2024 · W11 Pro · Specs según albarán renting (modelo 3540)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inventario: Caja 1 - Dell Latitude 3540 CKGYT04
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1001,6 +1001,55 @@
       <c r="K11" s="2" t="inlineStr">
         <is>
           <t>Service Tag 6ZLL214 · Express Code 15213264520 · Fab. 2024 · W11 Pro · Specs según albarán renting (modelo 3540)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Dell</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Latitude 3540 (Reg. P170G)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>CKGYT04</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Intel Core i7-1355U</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>512 GB SSD</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>15,6"</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Service Tag CKGYT04 · Express Code 27359209300 · Fab. 2024 · W11 Pro · Specs según albarán renting (modelo 3540)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inventario: Caja 2 - Dell Latitude 3550 6WDBX14
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1050,6 +1050,55 @@
       <c r="K12" s="2" t="inlineStr">
         <is>
           <t>Service Tag CKGYT04 · Express Code 27359209300 · Fab. 2024 · W11 Pro · Specs según albarán renting (modelo 3540)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Dell</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Latitude 3550 (Reg. P170G)</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>6WDBX14</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Intel Core i7-1355U (13ª gen)</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>512 GB SSD NVMe</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>15,6"</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Service Tag 6WDBX14 · Express Code 15018002680 · Fab. 2024 · Specs según indicación (igual que 3WDBX14)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inventario: Caja 2 - Dell Latitude 3540 1XLL214
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1099,6 +1099,55 @@
       <c r="K13" s="2" t="inlineStr">
         <is>
           <t>Service Tag 6WDBX14 · Express Code 15018002680 · Fab. 2024 · Specs según indicación (igual que 3WDBX14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Dell</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Latitude 3540 (Reg. P170G)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>1XLL214</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Intel Core i7-1355U</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>512 GB SSD</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>15,6"</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Service Tag 1XLL214 · Express Code 4208420488 · Fab. 2024 · W11 Pro · Specs según albarán renting (modelo 3540)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inventario: Renting - Dell Latitude 3540 2SLVMX3
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1148,6 +1148,57 @@
       <c r="K14" s="2" t="inlineStr">
         <is>
           <t>Service Tag 1XLL214 · Express Code 4208420488 · Fab. 2024 · W11 Pro · Specs según albarán renting (modelo 3540)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Renting</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Dell</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Latitude 3540 (Reg. P170G)</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>2SLVMX3</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Intel Core i7-1355U</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>512 GB SSD</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>15,6"</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Service Tag 2SLVMX3 · Express Code 6083365575 · Fab. 2023 · W11 Pro · EN LISTA RENTING</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inventario: Renting - Dell Latitude 3540 1VLVMX3
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1199,6 +1199,57 @@
       <c r="K15" s="2" t="inlineStr">
         <is>
           <t>Service Tag 2SLVMX3 · Express Code 6083365575 · Fab. 2023 · W11 Pro · EN LISTA RENTING</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Renting</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Dell</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Latitude 3540 (Reg. P170G)</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>1VLVMX3</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Intel Core i7-1355U</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>512 GB SSD</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>15,6"</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Service Tag 1VLVMX3 · Express Code 4087981767 · Fab. 2023 · W11 Pro · EN LISTA RENTING</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inventario: Caja 2 - Dell Latitude 3550 C0FBX14
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1250,6 +1250,55 @@
       <c r="K16" s="2" t="inlineStr">
         <is>
           <t>Service Tag 1VLVMX3 · Express Code 4087981767 · Fab. 2023 · W11 Pro · EN LISTA RENTING</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Dell</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Latitude 3550 (Reg. P170G)</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>C0FBX14</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Intel Core i7-1355U (13ª gen)</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>512 GB SSD NVMe</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>15,6"</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Service Tag C0FBX14 (con cero) · Express Code 26147138296 · Fab. 2024 · Specs según indicación (igual que 3WDBX14)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inventario: Caja 2 - Dell Latitude 3540 HYLL214
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1299,6 +1299,55 @@
       <c r="K17" s="2" t="inlineStr">
         <is>
           <t>Service Tag C0FBX14 (con cero) · Express Code 26147138296 · Fab. 2024 · Specs según indicación (igual que 3WDBX14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Dell</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Latitude 3540 (Reg. P170G)</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>HYLL214</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Intel Core i7-1355U</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>512 GB SSD</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>15,6"</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Service Tag HYLL214 · Express Code 39097404040 · Fab. 2024 · W11 Pro · Specs según albarán renting (modelo 3540)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inventario: Caja 2 - Dell Latitude 3540 FXLL214
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1348,6 +1348,55 @@
       <c r="K18" s="2" t="inlineStr">
         <is>
           <t>Service Tag HYLL214 · Express Code 39097404040 · Fab. 2024 · W11 Pro · Specs según albarán renting (modelo 3540)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Dell</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Latitude 3540 (Reg. P170G)</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>FXLL214</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Intel Core i7-1355U</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>512 GB SSD</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>15,6"</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Service Tag FXLL214 · Express Code 34683373192 · Fab. 2024 · W11 Pro · Specs según albarán renting (modelo 3540)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inventario: Caja 2 - Dell Latitude 3540 7YLL214
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1397,6 +1397,55 @@
       <c r="K19" s="2" t="inlineStr">
         <is>
           <t>Service Tag FXLL214 · Express Code 34683373192 · Fab. 2024 · W11 Pro · Specs según albarán renting (modelo 3540)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Dell</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Latitude 3540 (Reg. P170G)</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>7YLL214</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Intel Core i7-1355U</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>512 GB SSD</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>15,6"</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Service Tag 7YLL214 · Express Code 17329580680 · Fab. 2024 · W11 Pro · Specs según albarán renting (modelo 3540)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inventario: Caja 2 - Dell Latitude 3540 9YLL214
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1446,6 +1446,55 @@
       <c r="K20" s="2" t="inlineStr">
         <is>
           <t>Service Tag 7YLL214 · Express Code 17329580680 · Fab. 2024 · W11 Pro · Specs según albarán renting (modelo 3540)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Dell</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Latitude 3540 (Reg. P170G)</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>9YLL214</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Intel Core i7-1355U</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>512 GB SSD</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>15,6"</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Service Tag 9YLL214 · Express Code 21683145352 · Fab. 2024 · W11 Pro · Specs según albarán renting (modelo 3540)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Lista renting: añadir 8ZLL214
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -1509,7 +1509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1610,7 +1610,20 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>8ZLL214</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Indicado por el usuario (no estaba en el albarán)</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Nota: en la captura '1MS1KX3' y '4JS1KX3' podrían leerse con 5 en vez de S (1M51KX3 / 4J51KX3).</t>
         </is>

</xml_diff>

<commit_message>
Lista renting: quitar 8ZLL214
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -1509,7 +1509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1610,20 +1610,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>8ZLL214</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Indicado por el usuario (no estaba en el albarán)</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Nota: en la captura '1MS1KX3' y '4JS1KX3' podrían leerse con 5 en vez de S (1M51KX3 / 4J51KX3).</t>
         </is>

</xml_diff>

<commit_message>
Inventario: Renting - Latitude 3540 4J51KX3, pantalla rota
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00 €"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,8 +36,13 @@
     <font>
       <name val="Arial"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -47,6 +52,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE699"/>
       </patternFill>
     </fill>
   </fills>
@@ -62,7 +72,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -70,6 +80,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1495,6 +1506,61 @@
       <c r="K21" s="2" t="inlineStr">
         <is>
           <t>Service Tag 9YLL214 · Express Code 21683145352 · Fab. 2024 · W11 Pro · Specs según albarán renting (modelo 3540)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Renting</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Dell</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Latitude 3540 (Reg. P170G)</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>4J51KX3</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Intel Core i7-1355U</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>512 GB SSD</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>15,6"</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>PANTALLA ROTA – PARA REPARAR</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Service Tag 4J51KX3 · Express Code 9864458535 · Fab. 2023 · W11 Pro · EN LISTA RENTING</t>
         </is>
       </c>
     </row>
@@ -1552,7 +1618,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>1MS1KX3</t>
+          <t>1M51KX3</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -1597,7 +1663,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>4JS1KX3</t>
+          <t>4J51KX3</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -1612,7 +1678,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Nota: en la captura '1MS1KX3' y '4JS1KX3' podrían leerse con 5 en vez de S (1M51KX3 / 4J51KX3).</t>
+          <t>Nota: confirmado con la pegatina que 4J51KX3 lleva un 5 (no S); 1M51KX3 se ha corregido igual por el mismo patrón.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Añadir lista de equipos para reparar
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventario" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lista Renting" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lista Reparación" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1685,4 +1686,112 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Nº de serie</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Avería</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Estado en inventario</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>4J51KX3</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Dell Latitude 3540</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Pantalla rota</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Registrado (caja Renting)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>CND1505VK1</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>HP 250 G8 (RTL8822CE)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>No enciende</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente de aparecer</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>5CD947846T</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>HP Pavilion</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Pantalla rota</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente de aparecer</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Inventario: Caja 2 - Dell Vostro 8CVWZQ3 y Avell A55 MOB
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1562,6 +1562,72 @@
       <c r="K22" s="2" t="inlineStr">
         <is>
           <t>Service Tag 4J51KX3 · Express Code 9864458535 · Fab. 2023 · W11 Pro · EN LISTA RENTING</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Dell</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Vostro (modelo exacto pendiente)</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>8CVWZQ3</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Service Tag 8CVWZQ3 · Express Code 18193460187 · Fabricado en Brasil · Pegatina Windows · FALTA: modelo, CPU, RAM, disco</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Avell</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>A55 MOB</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>AVNB22180186</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>GPU NVIDIA GTX 1650 · Fabricado en Manaus (Brasil) · Etiqueta patrimonio Stilingue 001200 · FALTA: CPU, RAM, disco</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inventario: Caja 2 - HP 250 G8 CND1505VK1 (no enciende)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1628,6 +1628,47 @@
       <c r="K24" s="2" t="inlineStr">
         <is>
           <t>GPU NVIDIA GTX 1650 · Fabricado en Manaus (Brasil) · Etiqueta patrimonio Stilingue 001200 · FALTA: CPU, RAM, disco</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>250 G8 (ProdID 4K806EA#ABE)</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>CND1505VK1</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr"/>
+      <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>15,6"</t>
+        </is>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>NO ENCIENDE – PARA REPARAR</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Wi-Fi Realtek RTL8822CE · Garantía 1/1/0 · Etiqueta inventario 08178 · EN LISTA REPARACIÓN · FALTA: CPU, RAM, disco</t>
         </is>
       </c>
     </row>
@@ -1831,7 +1872,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Pendiente de aparecer</t>
+          <t>Registrado (Caja 2)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inventario: Caja 2 - HP 250 G8 CND1505VF4 y HP Pavilion 5CD947846T (pantalla rota)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1669,6 +1669,84 @@
       <c r="K25" s="2" t="inlineStr">
         <is>
           <t>Wi-Fi Realtek RTL8822CE · Garantía 1/1/0 · Etiqueta inventario 08178 · EN LISTA REPARACIÓN · FALTA: CPU, RAM, disco</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>250 G8 (ProdID 4K806EA#ABE)</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>CND1505VF4</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>15,6"</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Wi-Fi Realtek RTL8822CE · Garantía 1/1/0 · Pegatina Windows · Mismo lote que CND1505VK1 (este NO está en reparación) · FALTA: CPU, RAM, disco</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Pavilion 14-ce3009ns (ProdID 8PN56EA#ABE)</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>5CD947846T</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>14"</t>
+        </is>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>PANTALLA ROTA – PARA REPARAR</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Wi-Fi Intel 9560NGW · Garantía 1/1/0 · EN LISTA REPARACIÓN · FALTA: CPU, RAM, disco (confirmar)</t>
         </is>
       </c>
     </row>
@@ -1894,7 +1972,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Pendiente de aparecer</t>
+          <t>Registrado (Caja 2)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cerrar Caja 2: etiqueta PDF, reparaciones fuera de caja, HP a Caja 3
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -1635,8 +1635,10 @@
       <c r="A25" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="2" t="n">
-        <v>2</v>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Reparación (fuera de caja)</t>
+        </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
@@ -1677,7 +1679,7 @@
         <v>25</v>
       </c>
       <c r="B26" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
@@ -1713,8 +1715,10 @@
       <c r="A27" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="2" t="n">
-        <v>2</v>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Reparación (fuera de caja)</t>
+        </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
@@ -1950,7 +1954,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Registrado (Caja 2)</t>
+          <t>Registrado (fuera de caja, para reparar)</t>
         </is>
       </c>
     </row>
@@ -1972,7 +1976,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Registrado (Caja 2)</t>
+          <t>Registrado (fuera de caja, para reparar)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inventario: Caja 3 - HP Pavilion x360 5CG104310F
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1751,6 +1751,43 @@
       <c r="K27" s="2" t="inlineStr">
         <is>
           <t>Wi-Fi Intel 9560NGW · Garantía 1/1/0 · EN LISTA REPARACIÓN · FALTA: CPU, RAM, disco (confirmar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Pavilion x360 Convertible 14-dw1020ns (ProdID 27S62EA#ABE)</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>5CG104310F</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr"/>
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>14" táctil convertible</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Wi-Fi Intel AX201NGW · Garantía 1/1/0 · Nº serie leído de grabado en carcasa (confirmar 0 vs O) · FALTA: CPU, RAM, disco</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inventario: Caja 3 - HP Pavilion x360 5CG10430PX
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1787,7 +1787,44 @@
       <c r="J28" s="2" t="inlineStr"/>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>Wi-Fi Intel AX201NGW · Garantía 1/1/0 · Nº serie leído de grabado en carcasa (confirmar 0 vs O) · FALTA: CPU, RAM, disco</t>
+          <t>Wi-Fi Intel AX201NGW · Garantía 1/1/0 · Nº serie confirmado por el usuario (cero) · FALTA: CPU, RAM, disco</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Pavilion x360 Convertible 14-dw1020ns (ProdID 27S62EA#ABE)</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>5CG10430PX</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr"/>
+      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>14" táctil convertible</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Wi-Fi Intel AX201NGW · Garantía 1/1/0 · FALTA: CPU, RAM, disco</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inventario: Caja 3 - Dell Vostro 3520 67JCBV3
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1825,6 +1825,43 @@
       <c r="K29" s="2" t="inlineStr">
         <is>
           <t>Wi-Fi Intel AX201NGW · Garantía 1/1/0 · FALTA: CPU, RAM, disco</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Dell</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Vostro 3520 (Reg. P112F)</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>67JCBV3</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr"/>
+      <c r="G30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>15,6"</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Service Tag 67JCBV3 · Express Code 13516445199 · Fabricado en Brasil · Wi-Fi AX201NGW · FALTA: CPU, RAM, disco</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inventario: Caja 3 - MacBook Air M1 C02JMC43Q6L4
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K30"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1862,6 +1862,47 @@
       <c r="K30" s="2" t="inlineStr">
         <is>
           <t>Service Tag 67JCBV3 · Express Code 13516445199 · Fabricado en Brasil · Wi-Fi AX201NGW · FALTA: CPU, RAM, disco</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>MacBook Air (M1, 2020) – A2337</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>C02JMC43Q6L4</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Apple M1</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr"/>
+      <c r="H31" s="2" t="inlineStr"/>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>13,3"</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Model A2337 · EMC 3598 · Gris espacial · FALTA: RAM (8/16 GB), almacenamiento; comprobar que no tiene bloqueo de iCloud/Buscar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inventario: Caja 3 - 2x MacBook Pro 13 M1
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1903,6 +1903,88 @@
       <c r="K31" s="2" t="inlineStr">
         <is>
           <t>Model A2337 · EMC 3598 · Gris espacial · FALTA: RAM (8/16 GB), almacenamiento; comprobar que no tiene bloqueo de iCloud/Buscar</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>MacBook Pro 13" (M1, 2020) – A2338</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>C02DX8YKQ05D</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Apple M1</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>13,3"</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr"/>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Model A2338 · EMC 3578 · Gris espacial · FALTA: RAM (8/16 GB), almacenamiento; comprobar que no tiene bloqueo de iCloud/Buscar</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>MacBook Pro 13" (M1, 2020) – A2338</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>C02DWF3CQ05D</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Apple M1</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="inlineStr"/>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>13,3"</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Model A2338 · EMC 3578 · Gris espacial · FALTA: RAM (8/16 GB), almacenamiento; comprobar que no tiene bloqueo de iCloud/Buscar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inventario: Caja 3 - Microsoft Surface Laptop (serie pendiente)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1985,6 +1985,39 @@
       <c r="K33" s="2" t="inlineStr">
         <is>
           <t>Model A2338 · EMC 3578 · Gris espacial · FALTA: RAM (8/16 GB), almacenamiento; comprobar que no tiene bloqueo de iCloud/Buscar</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Surface Laptop (modelo exacto pendiente)</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>PENDIENTE (ilegible en foto)</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr"/>
+      <c r="G34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr"/>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>Negro mate · Etiqueta Telcel/Radiomóvil Dipsa 'EQ. EXT 10124B' (quitar antes de vender) · FALTA: nº serie, modelo, CPU, RAM, disco</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inventario: Surface Laptop pantalla rota, fuera de caja
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -1992,8 +1992,10 @@
       <c r="A34" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="2" t="n">
-        <v>3</v>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Reparación (fuera de caja)</t>
+        </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
@@ -2014,7 +2016,11 @@
       <c r="G34" s="2" t="inlineStr"/>
       <c r="H34" s="2" t="inlineStr"/>
       <c r="I34" s="2" t="inlineStr"/>
-      <c r="J34" s="2" t="inlineStr"/>
+      <c r="J34" s="5" t="inlineStr">
+        <is>
+          <t>PANTALLA ROTA – PARA REPARAR</t>
+        </is>
+      </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
           <t>Negro mate · Etiqueta Telcel/Radiomóvil Dipsa 'EQ. EXT 10124B' (quitar antes de vender) · FALTA: nº serie, modelo, CPU, RAM, disco</t>
@@ -2150,7 +2156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2247,6 +2253,28 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft Surface Laptop</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Pantalla rota</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Registrado (fuera de caja, para reparar)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Inventario: Caja 3 - HP 250 G8 CND1505VF2
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:K35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2024,6 +2024,43 @@
       <c r="K34" s="2" t="inlineStr">
         <is>
           <t>Negro mate · Etiqueta Telcel/Radiomóvil Dipsa 'EQ. EXT 10124B' (quitar antes de vender) · FALTA: nº serie, modelo, CPU, RAM, disco</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>250 G8 (ProdID 4K806EA#ABE)</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>CND1505VF2</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>15,6"</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr"/>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>Wi-Fi Realtek RTL8822CE · Garantía 1/1/0 · Pegatina Windows · Etiqueta inventario 08179 · Mismo lote que CND1505VF4/VK1 · FALTA: CPU, RAM, disco</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inventario: Caja 4 - 8x MacBook Pro 14 M5 (verificados con albarán)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:K43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2061,6 +2061,430 @@
       <c r="K35" s="2" t="inlineStr">
         <is>
           <t>Wi-Fi Realtek RTL8822CE · Garantía 1/1/0 · Pegatina Windows · Etiqueta inventario 08179 · Mismo lote que CND1505VF4/VK1 · FALTA: CPU, RAM, disco</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>MacBook Pro 14" (M5, 2025) – A3434</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>GF06P6R4WK</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Apple M5 (10C CPU / 10C GPU)</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>1 TB SSD</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>14,2" Liquid Retina XDR</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo en caja</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>Part MDE54Y/A · Model A3434 · Plata · CPU 10 núcleos / GPU 10 núcleos · En caja de Apple · Nº serie leído de la caja · Verificado con albarán (16 uds, 8 en uso por usuarios)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>MacBook Pro 14" (M5, 2025) – A3434</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>KGRQ07KPY9</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Apple M5 (10C CPU / 10C GPU)</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>1 TB SSD</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>14,2" Liquid Retina XDR</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo en caja</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>Part MDE54Y/A · Model A3434 · Plata · CPU 10 núcleos / GPU 10 núcleos · En caja de Apple · Nº serie leído de la caja · Verificado con albarán (16 uds, 8 en uso por usuarios)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>MacBook Pro 14" (M5, 2025) – A3434</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>CNW661KH44</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Apple M5 (10C CPU / 10C GPU)</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>1 TB SSD</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>14,2" Liquid Retina XDR</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo en caja</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>Part MDE54Y/A · Model A3434 · Plata · CPU 10 núcleos / GPU 10 núcleos · En caja de Apple · Nº serie leído de la caja · Verificado con albarán (16 uds, 8 en uso por usuarios)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>MacBook Pro 14" (M5, 2025) – A3434</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>JC7PYQXVF4</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Apple M5 (10C CPU / 10C GPU)</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>1 TB SSD</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>14,2" Liquid Retina XDR</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo en caja</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>Part MDE54Y/A · Model A3434 · Plata · CPU 10 núcleos / GPU 10 núcleos · En caja de Apple · Nº serie leído de la caja · Verificado con albarán (16 uds, 8 en uso por usuarios)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>MacBook Pro 14" (M5, 2025) – A3434</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>C0DCQ2596Q</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Apple M5 (10C CPU / 10C GPU)</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>1 TB SSD</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>14,2" Liquid Retina XDR</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo en caja</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>Part MDE54Y/A · Model A3434 · Plata · CPU 10 núcleos / GPU 10 núcleos · En caja de Apple · Nº serie leído de la caja · Verificado con albarán (16 uds, 8 en uso por usuarios)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>MacBook Pro 14" (M5, 2025) – A3434</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>G46G6CHYFR</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Apple M5 (10C CPU / 10C GPU)</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>1 TB SSD</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>14,2" Liquid Retina XDR</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo en caja</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>Part MDE54Y/A · Model A3434 · Plata · CPU 10 núcleos / GPU 10 núcleos · En caja de Apple · Nº serie leído de la caja · Verificado con albarán (16 uds, 8 en uso por usuarios)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>MacBook Pro 14" (M5, 2025) – A3434</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>MH2JCJWRY1</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Apple M5 (10C CPU / 10C GPU)</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>1 TB SSD</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>14,2" Liquid Retina XDR</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo en caja</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>Part MDE54Y/A · Model A3434 · Plata · CPU 10 núcleos / GPU 10 núcleos · En caja de Apple · Nº serie leído de la caja · Verificado con albarán (16 uds, 8 en uso por usuarios)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>MacBook Pro 14" (M5, 2025) – A3434</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>C71KP6TGV9</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Apple M5 (10C CPU / 10C GPU)</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>1 TB SSD</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>14,2" Liquid Retina XDR</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo en caja</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>Part MDE54Y/A · Model A3434 · Plata · CPU 10 núcleos / GPU 10 núcleos · En caja de Apple · Nº serie leído de la caja · Verificado con albarán (16 uds, 8 en uso por usuarios)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inventario: completar características (internet + usuario) y regenerar etiquetas Caja 2 y 3
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -1587,14 +1587,26 @@
           <t>8CVWZQ3</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr"/>
-      <c r="G23" s="2" t="inlineStr"/>
-      <c r="H23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>SIN VERIFICAR</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>SIN VERIFICAR</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>SIN VERIFICAR</t>
+        </is>
+      </c>
       <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>Service Tag 8CVWZQ3 · Express Code 18193460187 · Fabricado en Brasil · Pegatina Windows · FALTA: modelo, CPU, RAM, disco</t>
+          <t>Service Tag 8CVWZQ3 · Express Code 18193460187 · Fabricado en Brasil · Pegatina Windows · Specs: sin modelo exacto ni datos; sin verificar</t>
         </is>
       </c>
     </row>
@@ -1620,14 +1632,26 @@
           <t>AVNB22180186</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr"/>
-      <c r="G24" s="2" t="inlineStr"/>
-      <c r="H24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Intel Core i5-11400H (probable) + GTX 1650</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>SIN VERIFICAR</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>SIN VERIFICAR</t>
+        </is>
+      </c>
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>GPU NVIDIA GTX 1650 · Fabricado en Manaus (Brasil) · Etiqueta patrimonio Stilingue 001200 · FALTA: CPU, RAM, disco</t>
+          <t>GPU NVIDIA GTX 1650 · Fabricado en Manaus (Brasil) · Etiqueta patrimonio Stilingue 001200 · Specs: CPU deducida del modelo A55 (internet); RAM/disco configurables, sin verificar</t>
         </is>
       </c>
     </row>
@@ -1655,9 +1679,21 @@
           <t>CND1505VK1</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr"/>
-      <c r="G25" s="2" t="inlineStr"/>
-      <c r="H25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Intel Core i5-1135G7</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>512 GB SSD NVMe</t>
+        </is>
+      </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
           <t>15,6"</t>
@@ -1670,7 +1706,7 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>Wi-Fi Realtek RTL8822CE · Garantía 1/1/0 · Etiqueta inventario 08178 · EN LISTA REPARACIÓN · FALTA: CPU, RAM, disco</t>
+          <t>Wi-Fi Realtek RTL8822CE · Garantía 1/1/0 · Etiqueta inventario 08178 · EN LISTA REPARACIÓN · Specs: ficha oficial del ProdID 4K806EA (internet); el usuario confirma i5</t>
         </is>
       </c>
     </row>
@@ -1696,9 +1732,21 @@
           <t>CND1505VF4</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr"/>
-      <c r="G26" s="2" t="inlineStr"/>
-      <c r="H26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Intel Core i5-1135G7</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>512 GB SSD NVMe</t>
+        </is>
+      </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
           <t>15,6"</t>
@@ -1707,7 +1755,7 @@
       <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>Wi-Fi Realtek RTL8822CE · Garantía 1/1/0 · Pegatina Windows · Mismo lote que CND1505VK1 (este NO está en reparación) · FALTA: CPU, RAM, disco</t>
+          <t>Wi-Fi Realtek RTL8822CE · Garantía 1/1/0 · Pegatina Windows · Mismo lote que CND1505VK1 (este NO está en reparación) · Specs: ficha oficial del ProdID 4K806EA (internet); el usuario confirma i5</t>
         </is>
       </c>
     </row>
@@ -1735,9 +1783,21 @@
           <t>5CD947846T</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr"/>
-      <c r="G27" s="2" t="inlineStr"/>
-      <c r="H27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Intel Core i5-1035G1 + NVIDIA MX130</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>1 TB SSD NVMe</t>
+        </is>
+      </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
           <t>14"</t>
@@ -1750,7 +1810,7 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>Wi-Fi Intel 9560NGW · Garantía 1/1/0 · EN LISTA REPARACIÓN · FALTA: CPU, RAM, disco (confirmar)</t>
+          <t>Wi-Fi Intel 9560NGW · Garantía 1/1/0 · EN LISTA REPARACIÓN · Specs: ficha oficial HP del ProdID 8PN56EA (internet)</t>
         </is>
       </c>
     </row>
@@ -1776,9 +1836,21 @@
           <t>5CG104310F</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr"/>
-      <c r="G28" s="2" t="inlineStr"/>
-      <c r="H28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Intel Core i5-1135G7</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>512 GB SSD NVMe</t>
+        </is>
+      </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
           <t>14" táctil convertible</t>
@@ -1787,7 +1859,7 @@
       <c r="J28" s="2" t="inlineStr"/>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>Wi-Fi Intel AX201NGW · Garantía 1/1/0 · Nº serie confirmado por el usuario (cero) · FALTA: CPU, RAM, disco</t>
+          <t>Wi-Fi Intel AX201NGW · Garantía 1/1/0 · Nº serie confirmado por el usuario (cero) · Specs: ficha oficial HP del ProdID 27S62EA (internet)</t>
         </is>
       </c>
     </row>
@@ -1813,9 +1885,21 @@
           <t>5CG10430PX</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr"/>
-      <c r="G29" s="2" t="inlineStr"/>
-      <c r="H29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Intel Core i5-1135G7</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>512 GB SSD NVMe</t>
+        </is>
+      </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
           <t>14" táctil convertible</t>
@@ -1824,7 +1908,7 @@
       <c r="J29" s="2" t="inlineStr"/>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>Wi-Fi Intel AX201NGW · Garantía 1/1/0 · FALTA: CPU, RAM, disco</t>
+          <t>Wi-Fi Intel AX201NGW · Garantía 1/1/0 · Specs: ficha oficial HP del ProdID 27S62EA (internet)</t>
         </is>
       </c>
     </row>
@@ -1850,9 +1934,21 @@
           <t>67JCBV3</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr"/>
-      <c r="G30" s="2" t="inlineStr"/>
-      <c r="H30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>SIN VERIFICAR</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>SIN VERIFICAR</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>SIN VERIFICAR</t>
+        </is>
+      </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
           <t>15,6"</t>
@@ -1861,7 +1957,7 @@
       <c r="J30" s="2" t="inlineStr"/>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>Service Tag 67JCBV3 · Express Code 13516445199 · Fabricado en Brasil · Wi-Fi AX201NGW · FALTA: CPU, RAM, disco</t>
+          <t>Service Tag 67JCBV3 · Express Code 13516445199 · Fabricado en Brasil · Wi-Fi AX201NGW · Specs: no se encuentra configuración fija del modelo brasileño P112F; sin verificar</t>
         </is>
       </c>
     </row>
@@ -1892,8 +1988,16 @@
           <t>Apple M1</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr"/>
-      <c r="H31" s="2" t="inlineStr"/>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>8 GB</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>256 GB SSD</t>
+        </is>
+      </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
           <t>13,3"</t>
@@ -1902,7 +2006,7 @@
       <c r="J31" s="2" t="inlineStr"/>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>Model A2337 · EMC 3598 · Gris espacial · FALTA: RAM (8/16 GB), almacenamiento; comprobar que no tiene bloqueo de iCloud/Buscar</t>
+          <t>Model A2337 · EMC 3598 · Gris espacial · comprobar que no tiene bloqueo de iCloud/Buscar · Specs: indicado por el usuario</t>
         </is>
       </c>
     </row>
@@ -1933,8 +2037,16 @@
           <t>Apple M1</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr"/>
-      <c r="H32" s="2" t="inlineStr"/>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>8 GB</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>256 GB SSD</t>
+        </is>
+      </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
           <t>13,3"</t>
@@ -1943,7 +2055,7 @@
       <c r="J32" s="2" t="inlineStr"/>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>Model A2338 · EMC 3578 · Gris espacial · FALTA: RAM (8/16 GB), almacenamiento; comprobar que no tiene bloqueo de iCloud/Buscar</t>
+          <t>Model A2338 · EMC 3578 · Gris espacial · comprobar que no tiene bloqueo de iCloud/Buscar · Specs: indicado por el usuario</t>
         </is>
       </c>
     </row>
@@ -1974,8 +2086,16 @@
           <t>Apple M1</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr"/>
-      <c r="H33" s="2" t="inlineStr"/>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>8 GB</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>256 GB SSD</t>
+        </is>
+      </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
           <t>13,3"</t>
@@ -1984,7 +2104,7 @@
       <c r="J33" s="2" t="inlineStr"/>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>Model A2338 · EMC 3578 · Gris espacial · FALTA: RAM (8/16 GB), almacenamiento; comprobar que no tiene bloqueo de iCloud/Buscar</t>
+          <t>Model A2338 · EMC 3578 · Gris espacial · comprobar que no tiene bloqueo de iCloud/Buscar · Specs: indicado por el usuario</t>
         </is>
       </c>
     </row>
@@ -2012,9 +2132,21 @@
           <t>PENDIENTE (ilegible en foto)</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr"/>
-      <c r="G34" s="2" t="inlineStr"/>
-      <c r="H34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>SIN VERIFICAR</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>SIN VERIFICAR</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>SIN VERIFICAR</t>
+        </is>
+      </c>
       <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="5" t="inlineStr">
         <is>
@@ -2023,7 +2155,7 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>Negro mate · Etiqueta Telcel/Radiomóvil Dipsa 'EQ. EXT 10124B' (quitar antes de vender) · FALTA: nº serie, modelo, CPU, RAM, disco</t>
+          <t>Negro mate · Etiqueta Telcel/Radiomóvil Dipsa 'EQ. EXT 10124B' (quitar antes de vender) · FALTA: nº serie · Specs: sin nº serie ni datos; sin verificar</t>
         </is>
       </c>
     </row>
@@ -2049,9 +2181,21 @@
           <t>CND1505VF2</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr"/>
-      <c r="G35" s="2" t="inlineStr"/>
-      <c r="H35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Intel Core i5-1135G7</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>16 GB</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>512 GB SSD NVMe</t>
+        </is>
+      </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
           <t>15,6"</t>
@@ -2060,7 +2204,7 @@
       <c r="J35" s="2" t="inlineStr"/>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>Wi-Fi Realtek RTL8822CE · Garantía 1/1/0 · Pegatina Windows · Etiqueta inventario 08179 · Mismo lote que CND1505VF4/VK1 · FALTA: CPU, RAM, disco</t>
+          <t>Wi-Fi Realtek RTL8822CE · Garantía 1/1/0 · Pegatina Windows · Etiqueta inventario 08179 · Mismo lote que CND1505VF4/VK1 · Specs: ficha oficial del ProdID 4K806EA (internet); el usuario confirma i5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inventario: Avell 16 GB / 512 GB
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmvdXFqYxnwRDH8tVmC7yv
</commit_message>
<xml_diff>
--- a/inventario_portatiles.xlsx
+++ b/inventario_portatiles.xlsx
@@ -1639,19 +1639,19 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>SIN VERIFICAR</t>
+          <t>16 GB</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>SIN VERIFICAR</t>
+          <t>512 GB SSD</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>GPU NVIDIA GTX 1650 · Fabricado en Manaus (Brasil) · Etiqueta patrimonio Stilingue 001200 · Specs: CPU deducida del modelo A55 (internet); RAM/disco configurables, sin verificar</t>
+          <t>GPU NVIDIA GTX 1650 · Fabricado en Manaus (Brasil) · Etiqueta patrimonio Stilingue 001200 · Specs: CPU deducida del modelo A55 (internet); RAM 16 GB y disco 512 GB indicados por el usuario</t>
         </is>
       </c>
     </row>

</xml_diff>